<commit_message>
Fixed month selection and dashboard updates
</commit_message>
<xml_diff>
--- a/data/Budget Tracker Final...xlsx
+++ b/data/Budget Tracker Final...xlsx
@@ -10938,7 +10938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.2"/>
   <cols>
     <col width="11.88671875" customWidth="1" style="53" min="1" max="1"/>
@@ -12185,7 +12185,6 @@
       <c r="E34" t="n">
         <v>1000</v>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
         <v>0.99</v>
       </c>
@@ -12195,6 +12194,361 @@
         </is>
       </c>
       <c r="I34" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pizza Hut</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>500</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Pizza and garlic bread</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>900</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Salary Recieved</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Bus ticket</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Loan</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>100</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Salary Recieved</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Bus Ticket</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Recieved from Parents</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>16-07-2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>2026</v>
       </c>
     </row>

</xml_diff>